<commit_message>
Update results of 365 of 1,144 files done (up to Ionosphere)
</commit_message>
<xml_diff>
--- a/results/Table-NRMS-AE_C10.xlsx
+++ b/results/Table-NRMS-AE_C10.xlsx
@@ -1817,6 +1817,14 @@
           <t>Glass_AE_5</t>
         </is>
       </c>
+      <c r="B95" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1824,6 +1832,14 @@
           <t>Glass_AE_10</t>
         </is>
       </c>
+      <c r="B96" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1831,6 +1847,14 @@
           <t>Glass_AE_20</t>
         </is>
       </c>
+      <c r="B97" t="n">
+        <v>0.0116</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1838,6 +1862,14 @@
           <t>Glass_AG_1</t>
         </is>
       </c>
+      <c r="B98" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1845,6 +1877,14 @@
           <t>Glass_AG_5</t>
         </is>
       </c>
+      <c r="B99" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1852,6 +1892,14 @@
           <t>Glass_AG_10</t>
         </is>
       </c>
+      <c r="B100" t="n">
+        <v>0.0067</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1859,6 +1907,14 @@
           <t>Glass_AG_20</t>
         </is>
       </c>
+      <c r="B101" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1866,6 +1922,14 @@
           <t>Glass_AL_1</t>
         </is>
       </c>
+      <c r="B102" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1873,6 +1937,14 @@
           <t>Glass_AL_5</t>
         </is>
       </c>
+      <c r="B103" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1880,6 +1952,14 @@
           <t>Glass_AL_10</t>
         </is>
       </c>
+      <c r="B104" t="n">
+        <v>0.0057</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1887,6 +1967,14 @@
           <t>Glass_AL_20</t>
         </is>
       </c>
+      <c r="B105" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1894,6 +1982,14 @@
           <t>Glass_AN_1</t>
         </is>
       </c>
+      <c r="B106" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1901,6 +1997,14 @@
           <t>Glass_AN_5</t>
         </is>
       </c>
+      <c r="B107" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1908,6 +2012,14 @@
           <t>Glass_AN_10</t>
         </is>
       </c>
+      <c r="B108" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1915,6 +2027,14 @@
           <t>Glass_AN_20</t>
         </is>
       </c>
+      <c r="B109" t="n">
+        <v>0.0157</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1922,6 +2042,14 @@
           <t>Glass_AW_1</t>
         </is>
       </c>
+      <c r="B110" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1929,6 +2057,14 @@
           <t>Glass_AW_5</t>
         </is>
       </c>
+      <c r="B111" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1936,6 +2072,14 @@
           <t>Glass_AW_10</t>
         </is>
       </c>
+      <c r="B112" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1943,6 +2087,14 @@
           <t>Glass_AW_20</t>
         </is>
       </c>
+      <c r="B113" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1950,6 +2102,14 @@
           <t>Glass_NE_1</t>
         </is>
       </c>
+      <c r="B114" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1957,6 +2117,14 @@
           <t>Glass_NE_5</t>
         </is>
       </c>
+      <c r="B115" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1964,6 +2132,14 @@
           <t>Glass_NE_10</t>
         </is>
       </c>
+      <c r="B116" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1971,6 +2147,14 @@
           <t>Glass_NE_20</t>
         </is>
       </c>
+      <c r="B117" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1978,6 +2162,14 @@
           <t>Glass_NG_1</t>
         </is>
       </c>
+      <c r="B118" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1985,6 +2177,14 @@
           <t>Glass_NG_5</t>
         </is>
       </c>
+      <c r="B119" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1992,6 +2192,14 @@
           <t>Glass_NG_10</t>
         </is>
       </c>
+      <c r="B120" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1999,6 +2207,14 @@
           <t>Glass_NG_20</t>
         </is>
       </c>
+      <c r="B121" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2006,6 +2222,14 @@
           <t>Glass_NL_1</t>
         </is>
       </c>
+      <c r="B122" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2013,6 +2237,14 @@
           <t>Glass_NL_5</t>
         </is>
       </c>
+      <c r="B123" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2020,6 +2252,14 @@
           <t>Glass_NL_10</t>
         </is>
       </c>
+      <c r="B124" t="n">
+        <v>0.0073</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2027,6 +2267,14 @@
           <t>Glass_NL_20</t>
         </is>
       </c>
+      <c r="B125" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2034,6 +2282,14 @@
           <t>Glass_NN_1</t>
         </is>
       </c>
+      <c r="B126" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2041,6 +2297,14 @@
           <t>Glass_NN_5</t>
         </is>
       </c>
+      <c r="B127" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2048,6 +2312,14 @@
           <t>Glass_NN_10</t>
         </is>
       </c>
+      <c r="B128" t="n">
+        <v>0.0055</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2055,6 +2327,14 @@
           <t>Glass_NN_20</t>
         </is>
       </c>
+      <c r="B129" t="n">
+        <v>0.0106</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2062,6 +2342,14 @@
           <t>Glass_NW_1</t>
         </is>
       </c>
+      <c r="B130" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2069,6 +2357,14 @@
           <t>Glass_NW_5</t>
         </is>
       </c>
+      <c r="B131" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2076,6 +2372,14 @@
           <t>Glass_NW_10</t>
         </is>
       </c>
+      <c r="B132" t="n">
+        <v>0.0073</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2083,6 +2387,14 @@
           <t>Glass_NW_20</t>
         </is>
       </c>
+      <c r="B133" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2090,6 +2402,14 @@
           <t>Sheart_C_1</t>
         </is>
       </c>
+      <c r="B134" t="n">
+        <v>0.0236</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2097,6 +2417,14 @@
           <t>Sheart_C_5</t>
         </is>
       </c>
+      <c r="B135" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2104,6 +2432,14 @@
           <t>Sheart_C_10</t>
         </is>
       </c>
+      <c r="B136" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2111,6 +2447,14 @@
           <t>Sheart_C_20</t>
         </is>
       </c>
+      <c r="B137" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2118,6 +2462,14 @@
           <t>Sheart_AE_1</t>
         </is>
       </c>
+      <c r="B138" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2125,6 +2477,14 @@
           <t>Sheart_AE_5</t>
         </is>
       </c>
+      <c r="B139" t="n">
+        <v>0.0272</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2132,6 +2492,14 @@
           <t>Sheart_AE_10</t>
         </is>
       </c>
+      <c r="B140" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2139,6 +2507,14 @@
           <t>Sheart_AE_20</t>
         </is>
       </c>
+      <c r="B141" t="n">
+        <v>0.0707</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2146,6 +2522,14 @@
           <t>Sheart_AG_1</t>
         </is>
       </c>
+      <c r="B142" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2153,6 +2537,14 @@
           <t>Sheart_AG_5</t>
         </is>
       </c>
+      <c r="B143" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2160,6 +2552,14 @@
           <t>Sheart_AG_10</t>
         </is>
       </c>
+      <c r="B144" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2167,6 +2567,14 @@
           <t>Sheart_AG_20</t>
         </is>
       </c>
+      <c r="B145" t="n">
+        <v>0.0857</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2174,6 +2582,14 @@
           <t>Sheart_AL_1</t>
         </is>
       </c>
+      <c r="B146" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2181,6 +2597,14 @@
           <t>Sheart_AL_5</t>
         </is>
       </c>
+      <c r="B147" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2188,6 +2612,14 @@
           <t>Sheart_AL_10</t>
         </is>
       </c>
+      <c r="B148" t="n">
+        <v>0.0419</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2195,6 +2627,14 @@
           <t>Sheart_AL_20</t>
         </is>
       </c>
+      <c r="B149" t="n">
+        <v>0.0883</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2202,6 +2642,14 @@
           <t>Sheart_AN_1</t>
         </is>
       </c>
+      <c r="B150" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2209,6 +2657,14 @@
           <t>Sheart_AN_5</t>
         </is>
       </c>
+      <c r="B151" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2216,6 +2672,14 @@
           <t>Sheart_AN_10</t>
         </is>
       </c>
+      <c r="B152" t="n">
+        <v>0.0369</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2223,6 +2687,14 @@
           <t>Sheart_AN_20</t>
         </is>
       </c>
+      <c r="B153" t="n">
+        <v>0.07049999999999999</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2230,6 +2702,14 @@
           <t>Sheart_AW_1</t>
         </is>
       </c>
+      <c r="B154" t="n">
+        <v>0.0083</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2237,6 +2717,14 @@
           <t>Sheart_AW_5</t>
         </is>
       </c>
+      <c r="B155" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2244,6 +2732,14 @@
           <t>Sheart_AW_10</t>
         </is>
       </c>
+      <c r="B156" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2251,6 +2747,14 @@
           <t>Sheart_AW_20</t>
         </is>
       </c>
+      <c r="B157" t="n">
+        <v>0.0518</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2258,6 +2762,14 @@
           <t>Sheart_NE_1</t>
         </is>
       </c>
+      <c r="B158" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2265,6 +2777,14 @@
           <t>Sheart_NE_5</t>
         </is>
       </c>
+      <c r="B159" t="n">
+        <v>0.0512</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2272,6 +2792,14 @@
           <t>Sheart_NE_10</t>
         </is>
       </c>
+      <c r="B160" t="n">
+        <v>0.1033</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2279,6 +2807,14 @@
           <t>Sheart_NE_20</t>
         </is>
       </c>
+      <c r="B161" t="n">
+        <v>0.1153</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2286,6 +2822,14 @@
           <t>Sheart_NG_1</t>
         </is>
       </c>
+      <c r="B162" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2293,6 +2837,14 @@
           <t>Sheart_NG_5</t>
         </is>
       </c>
+      <c r="B163" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2300,6 +2852,14 @@
           <t>Sheart_NG_10</t>
         </is>
       </c>
+      <c r="B164" t="n">
+        <v>0.0696</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2307,6 +2867,14 @@
           <t>Sheart_NG_20</t>
         </is>
       </c>
+      <c r="B165" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2314,6 +2882,14 @@
           <t>Sheart_NL_1</t>
         </is>
       </c>
+      <c r="B166" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2321,6 +2897,14 @@
           <t>Sheart_NL_5</t>
         </is>
       </c>
+      <c r="B167" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2328,6 +2912,14 @@
           <t>Sheart_NL_10</t>
         </is>
       </c>
+      <c r="B168" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2335,6 +2927,14 @@
           <t>Sheart_NL_20</t>
         </is>
       </c>
+      <c r="B169" t="n">
+        <v>0.0977</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2342,6 +2942,14 @@
           <t>Sheart_NN_1</t>
         </is>
       </c>
+      <c r="B170" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2349,6 +2957,14 @@
           <t>Sheart_NN_5</t>
         </is>
       </c>
+      <c r="B171" t="n">
+        <v>0.0131</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2356,6 +2972,14 @@
           <t>Sheart_NN_10</t>
         </is>
       </c>
+      <c r="B172" t="n">
+        <v>0.0924</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2363,6 +2987,14 @@
           <t>Sheart_NN_20</t>
         </is>
       </c>
+      <c r="B173" t="n">
+        <v>0.0822</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2370,6 +3002,14 @@
           <t>Sheart_NW_1</t>
         </is>
       </c>
+      <c r="B174" t="n">
+        <v>0.0193</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2377,6 +3017,14 @@
           <t>Sheart_NW_5</t>
         </is>
       </c>
+      <c r="B175" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2384,6 +3032,14 @@
           <t>Sheart_NW_10</t>
         </is>
       </c>
+      <c r="B176" t="n">
+        <v>0.0682</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2391,6 +3047,14 @@
           <t>Sheart_NW_20</t>
         </is>
       </c>
+      <c r="B177" t="n">
+        <v>0.0862</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=500 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2398,6 +3062,14 @@
           <t>BUPA_C_1</t>
         </is>
       </c>
+      <c r="B178" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2405,6 +3077,14 @@
           <t>BUPA_C_5</t>
         </is>
       </c>
+      <c r="B179" t="n">
+        <v>0.0958</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2412,6 +3092,14 @@
           <t>BUPA_C_10</t>
         </is>
       </c>
+      <c r="B180" t="n">
+        <v>0.1028</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2419,6 +3107,14 @@
           <t>BUPA_C_20</t>
         </is>
       </c>
+      <c r="B181" t="n">
+        <v>0.1139</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2426,6 +3122,14 @@
           <t>BUPA_AE_1</t>
         </is>
       </c>
+      <c r="B182" t="n">
+        <v>0.0206</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2433,6 +3137,14 @@
           <t>BUPA_AE_5</t>
         </is>
       </c>
+      <c r="B183" t="n">
+        <v>0.06419999999999999</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2440,6 +3152,14 @@
           <t>BUPA_AE_10</t>
         </is>
       </c>
+      <c r="B184" t="n">
+        <v>0.0979</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2447,6 +3167,14 @@
           <t>BUPA_AE_20</t>
         </is>
       </c>
+      <c r="B185" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2454,6 +3182,14 @@
           <t>BUPA_AG_1</t>
         </is>
       </c>
+      <c r="B186" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2461,6 +3197,14 @@
           <t>BUPA_AG_5</t>
         </is>
       </c>
+      <c r="B187" t="n">
+        <v>0.0478</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2468,6 +3212,14 @@
           <t>BUPA_AG_10</t>
         </is>
       </c>
+      <c r="B188" t="n">
+        <v>0.1024</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2475,6 +3227,14 @@
           <t>BUPA_AG_20</t>
         </is>
       </c>
+      <c r="B189" t="n">
+        <v>0.1494</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2482,6 +3242,14 @@
           <t>BUPA_AL_1</t>
         </is>
       </c>
+      <c r="B190" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2489,6 +3257,14 @@
           <t>BUPA_AL_5</t>
         </is>
       </c>
+      <c r="B191" t="n">
+        <v>0.0762</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2496,6 +3272,14 @@
           <t>BUPA_AL_10</t>
         </is>
       </c>
+      <c r="B192" t="n">
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2503,6 +3287,14 @@
           <t>BUPA_AL_20</t>
         </is>
       </c>
+      <c r="B193" t="n">
+        <v>0.1607</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2510,6 +3302,14 @@
           <t>BUPA_AN_1</t>
         </is>
       </c>
+      <c r="B194" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2517,6 +3317,14 @@
           <t>BUPA_AN_5</t>
         </is>
       </c>
+      <c r="B195" t="n">
+        <v>0.08409999999999999</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2524,6 +3332,14 @@
           <t>BUPA_AN_10</t>
         </is>
       </c>
+      <c r="B196" t="n">
+        <v>0.1088</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2531,6 +3347,14 @@
           <t>BUPA_AN_20</t>
         </is>
       </c>
+      <c r="B197" t="n">
+        <v>0.1468</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2538,6 +3362,14 @@
           <t>BUPA_AW_1</t>
         </is>
       </c>
+      <c r="B198" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2545,6 +3377,14 @@
           <t>BUPA_AW_5</t>
         </is>
       </c>
+      <c r="B199" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2552,6 +3392,14 @@
           <t>BUPA_AW_10</t>
         </is>
       </c>
+      <c r="B200" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2559,6 +3407,14 @@
           <t>BUPA_AW_20</t>
         </is>
       </c>
+      <c r="B201" t="n">
+        <v>0.1473</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2566,6 +3422,14 @@
           <t>BUPA_NE_1</t>
         </is>
       </c>
+      <c r="B202" t="n">
+        <v>0.0252</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2573,6 +3437,14 @@
           <t>BUPA_NE_5</t>
         </is>
       </c>
+      <c r="B203" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2580,6 +3452,14 @@
           <t>BUPA_NE_10</t>
         </is>
       </c>
+      <c r="B204" t="n">
+        <v>0.09959999999999999</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2587,6 +3467,14 @@
           <t>BUPA_NE_20</t>
         </is>
       </c>
+      <c r="B205" t="n">
+        <v>0.1615</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2594,6 +3482,14 @@
           <t>BUPA_NG_1</t>
         </is>
       </c>
+      <c r="B206" t="n">
+        <v>0.0139</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2601,6 +3497,14 @@
           <t>BUPA_NG_5</t>
         </is>
       </c>
+      <c r="B207" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2608,6 +3512,14 @@
           <t>BUPA_NG_10</t>
         </is>
       </c>
+      <c r="B208" t="n">
+        <v>0.1225</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2615,6 +3527,14 @@
           <t>BUPA_NG_20</t>
         </is>
       </c>
+      <c r="B209" t="n">
+        <v>0.1345</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2622,6 +3542,14 @@
           <t>BUPA_NL_1</t>
         </is>
       </c>
+      <c r="B210" t="n">
+        <v>0.0109</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2629,6 +3557,14 @@
           <t>BUPA_NL_5</t>
         </is>
       </c>
+      <c r="B211" t="n">
+        <v>0.0487</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2636,6 +3572,14 @@
           <t>BUPA_NL_10</t>
         </is>
       </c>
+      <c r="B212" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2643,6 +3587,14 @@
           <t>BUPA_NL_20</t>
         </is>
       </c>
+      <c r="B213" t="n">
+        <v>0.1695</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2650,6 +3602,14 @@
           <t>BUPA_NN_1</t>
         </is>
       </c>
+      <c r="B214" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2657,6 +3617,14 @@
           <t>BUPA_NN_5</t>
         </is>
       </c>
+      <c r="B215" t="n">
+        <v>0.0485</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2664,6 +3632,14 @@
           <t>BUPA_NN_10</t>
         </is>
       </c>
+      <c r="B216" t="n">
+        <v>0.1442</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2671,6 +3647,14 @@
           <t>BUPA_NN_20</t>
         </is>
       </c>
+      <c r="B217" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2678,6 +3662,14 @@
           <t>BUPA_NW_1</t>
         </is>
       </c>
+      <c r="B218" t="n">
+        <v>0.0269</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2685,6 +3677,14 @@
           <t>BUPA_NW_5</t>
         </is>
       </c>
+      <c r="B219" t="n">
+        <v>0.0906</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2692,6 +3692,14 @@
           <t>BUPA_NW_10</t>
         </is>
       </c>
+      <c r="B220" t="n">
+        <v>0.0674</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2699,6 +3707,14 @@
           <t>BUPA_NW_20</t>
         </is>
       </c>
+      <c r="B221" t="n">
+        <v>0.1419</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2706,6 +3722,14 @@
           <t>Ionosphere_C_1</t>
         </is>
       </c>
+      <c r="B222" t="n">
+        <v>0.0585</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2713,6 +3737,14 @@
           <t>Ionosphere_C_5</t>
         </is>
       </c>
+      <c r="B223" t="n">
+        <v>0.1579</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2720,6 +3752,14 @@
           <t>Ionosphere_C_10</t>
         </is>
       </c>
+      <c r="B224" t="n">
+        <v>0.2014</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2727,6 +3767,14 @@
           <t>Ionosphere_C_20</t>
         </is>
       </c>
+      <c r="B225" t="n">
+        <v>0.3008</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2734,6 +3782,14 @@
           <t>Ionosphere_AE_1</t>
         </is>
       </c>
+      <c r="B226" t="n">
+        <v>0.0765</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2741,6 +3797,14 @@
           <t>Ionosphere_AE_5</t>
         </is>
       </c>
+      <c r="B227" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2748,6 +3812,14 @@
           <t>Ionosphere_AE_10</t>
         </is>
       </c>
+      <c r="B228" t="n">
+        <v>0.2384</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2755,6 +3827,14 @@
           <t>Ionosphere_AE_20</t>
         </is>
       </c>
+      <c r="B229" t="n">
+        <v>0.3512</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2762,6 +3842,14 @@
           <t>Ionosphere_AG_1</t>
         </is>
       </c>
+      <c r="B230" t="n">
+        <v>0.0635</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2769,6 +3857,14 @@
           <t>Ionosphere_AG_5</t>
         </is>
       </c>
+      <c r="B231" t="n">
+        <v>0.1394</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2776,6 +3872,14 @@
           <t>Ionosphere_AG_10</t>
         </is>
       </c>
+      <c r="B232" t="n">
+        <v>0.2273</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2783,6 +3887,14 @@
           <t>Ionosphere_AG_20</t>
         </is>
       </c>
+      <c r="B233" t="n">
+        <v>0.3428</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2790,6 +3902,14 @@
           <t>Ionosphere_AL_1</t>
         </is>
       </c>
+      <c r="B234" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=400 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3014,6 +4134,14 @@
           <t>Sonar_C_1</t>
         </is>
       </c>
+      <c r="B266" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3021,6 +4149,14 @@
           <t>Sonar_C_5</t>
         </is>
       </c>
+      <c r="B267" t="n">
+        <v>0.0474</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3028,6 +4164,14 @@
           <t>Sonar_C_10</t>
         </is>
       </c>
+      <c r="B268" t="n">
+        <v>0.07530000000000001</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3035,6 +4179,14 @@
           <t>Sonar_C_20</t>
         </is>
       </c>
+      <c r="B269" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3042,6 +4194,14 @@
           <t>Sonar_AE_1</t>
         </is>
       </c>
+      <c r="B270" t="n">
+        <v>0.0286</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3049,6 +4209,14 @@
           <t>Sonar_AE_5</t>
         </is>
       </c>
+      <c r="B271" t="n">
+        <v>0.0781</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3056,6 +4224,14 @@
           <t>Sonar_AE_10</t>
         </is>
       </c>
+      <c r="B272" t="n">
+        <v>0.1294</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3063,6 +4239,14 @@
           <t>Sonar_AE_20</t>
         </is>
       </c>
+      <c r="B273" t="n">
+        <v>0.1883</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3070,6 +4254,14 @@
           <t>Sonar_AG_1</t>
         </is>
       </c>
+      <c r="B274" t="n">
+        <v>0.0287</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3077,6 +4269,14 @@
           <t>Sonar_AG_5</t>
         </is>
       </c>
+      <c r="B275" t="n">
+        <v>0.0852</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3084,6 +4284,14 @@
           <t>Sonar_AG_10</t>
         </is>
       </c>
+      <c r="B276" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3091,6 +4299,14 @@
           <t>Sonar_AG_20</t>
         </is>
       </c>
+      <c r="B277" t="n">
+        <v>0.1955</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3098,6 +4314,14 @@
           <t>Sonar_AL_1</t>
         </is>
       </c>
+      <c r="B278" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3105,6 +4329,14 @@
           <t>Sonar_AL_5</t>
         </is>
       </c>
+      <c r="B279" t="n">
+        <v>0.0727</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3112,6 +4344,14 @@
           <t>Sonar_AL_10</t>
         </is>
       </c>
+      <c r="B280" t="n">
+        <v>0.1276</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3119,6 +4359,14 @@
           <t>Sonar_AL_20</t>
         </is>
       </c>
+      <c r="B281" t="n">
+        <v>0.1902</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3126,6 +4374,14 @@
           <t>Sonar_AN_1</t>
         </is>
       </c>
+      <c r="B282" t="n">
+        <v>0.0283</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3133,6 +4389,14 @@
           <t>Sonar_AN_5</t>
         </is>
       </c>
+      <c r="B283" t="n">
+        <v>0.0646</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3140,6 +4404,14 @@
           <t>Sonar_AN_10</t>
         </is>
       </c>
+      <c r="B284" t="n">
+        <v>0.1203</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3147,6 +4419,14 @@
           <t>Sonar_AN_20</t>
         </is>
       </c>
+      <c r="B285" t="n">
+        <v>0.1991</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3154,6 +4434,14 @@
           <t>Sonar_AW_1</t>
         </is>
       </c>
+      <c r="B286" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3161,6 +4449,14 @@
           <t>Sonar_AW_5</t>
         </is>
       </c>
+      <c r="B287" t="n">
+        <v>0.0718</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3168,6 +4464,14 @@
           <t>Sonar_AW_10</t>
         </is>
       </c>
+      <c r="B288" t="n">
+        <v>0.1274</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3175,6 +4479,14 @@
           <t>Sonar_AW_20</t>
         </is>
       </c>
+      <c r="B289" t="n">
+        <v>0.1948</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3182,6 +4494,14 @@
           <t>Sonar_NE_1</t>
         </is>
       </c>
+      <c r="B290" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3189,6 +4509,14 @@
           <t>Sonar_NE_5</t>
         </is>
       </c>
+      <c r="B291" t="n">
+        <v>0.0514</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3196,6 +4524,14 @@
           <t>Sonar_NE_10</t>
         </is>
       </c>
+      <c r="B292" t="n">
+        <v>0.0766</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3203,6 +4539,14 @@
           <t>Sonar_NE_20</t>
         </is>
       </c>
+      <c r="B293" t="n">
+        <v>0.1212</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3210,6 +4554,14 @@
           <t>Sonar_NG_1</t>
         </is>
       </c>
+      <c r="B294" t="n">
+        <v>0.0188</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3217,6 +4569,14 @@
           <t>Sonar_NG_5</t>
         </is>
       </c>
+      <c r="B295" t="n">
+        <v>0.0513</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3224,6 +4584,14 @@
           <t>Sonar_NG_10</t>
         </is>
       </c>
+      <c r="B296" t="n">
+        <v>0.07290000000000001</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3231,6 +4599,14 @@
           <t>Sonar_NG_20</t>
         </is>
       </c>
+      <c r="B297" t="n">
+        <v>0.1152</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3238,6 +4614,14 @@
           <t>Sonar_NL_1</t>
         </is>
       </c>
+      <c r="B298" t="n">
+        <v>0.0231</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3245,6 +4629,14 @@
           <t>Sonar_NL_5</t>
         </is>
       </c>
+      <c r="B299" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3252,6 +4644,14 @@
           <t>Sonar_NL_10</t>
         </is>
       </c>
+      <c r="B300" t="n">
+        <v>0.07829999999999999</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3259,6 +4659,14 @@
           <t>Sonar_NL_20</t>
         </is>
       </c>
+      <c r="B301" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3266,6 +4674,14 @@
           <t>Sonar_NN_1</t>
         </is>
       </c>
+      <c r="B302" t="n">
+        <v>0.0221</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3273,6 +4689,14 @@
           <t>Sonar_NN_5</t>
         </is>
       </c>
+      <c r="B303" t="n">
+        <v>0.0436</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3280,6 +4704,14 @@
           <t>Sonar_NN_10</t>
         </is>
       </c>
+      <c r="B304" t="n">
+        <v>0.0737</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3287,6 +4719,14 @@
           <t>Sonar_NN_20</t>
         </is>
       </c>
+      <c r="B305" t="n">
+        <v>0.1158</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3294,6 +4734,14 @@
           <t>Sonar_NW_1</t>
         </is>
       </c>
+      <c r="B306" t="n">
+        <v>0.0253</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3301,6 +4749,14 @@
           <t>Sonar_NW_5</t>
         </is>
       </c>
+      <c r="B307" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3308,11 +4764,27 @@
           <t>Sonar_NW_10</t>
         </is>
       </c>
+      <c r="B308" t="n">
+        <v>0.0791</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
           <t>Sonar_NW_20</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>0.1222</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>own VAEAC width=256 depth=4 latent=32 lr=0.0003 batch=64 hide p=0.2 epochs=667 K=25 seed=0</t>
         </is>
       </c>
     </row>

</xml_diff>